<commit_message>
Decisiones operador 2026-06-16: SG Antigüedad 104=4 + decisiones confirmadas
- datos_gobernanza.py: SG Antigüedad (104) 3 -> 4 (el Update NAIS may-2026 cuenta
  como estrategia vigente; decisión del operador). Regenerados PDF/xlsx/matriz md.
- Confirmadas y registradas (HANDOFF §3/§7): EU AI Act = iniciativa legal (128=3)
  en países UE; ERNC (145) = % renovables total (EMBER); patentes 83=país del
  solicitante / 84=país del inventor (resuelve el cruce de definiciones del Excel).
- Patentes: definición CPC + ventana = replicar ILIA 2025 (pendiente su spec);
  actualizado patentes_consultas_lens_espacenet.md (D1-D4) y la hoja Pendientes.
- Sin cambio de cobertura de color (138 verde / 21 ámbar / 31 rojo).

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
+++ b/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
@@ -1324,7 +1324,7 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>EE: White Paper 2024-30 · SG: NAIS 2.0 2023 · DE: Aktionsplan 2023 · ES: Estrategia 2024 · PT: ANIA 2026-30</t>
+          <t>EE: White Paper 2024-30 · SG: Update NAIS may-2026 = estrategia vigente (decisión operador) · DE: Aktionsplan 2023 · ES: Estrategia 2024 · PT: ANIA 2026-30</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Aplicantes e Inventores de patentes IA (83-84)</t>
+          <t>Aplicantes (83)=país del solicitante · Inventores (84)=país del inventor</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>NO existen en OECD.AI. Lens.org/Espacenet: CPC G06N facetado por país del SOLICITANTE / del INVENTOR.</t>
+          <t>NO existen en OECD.AI. Consultas listas en patentes_consultas_lens_espacenet.md (Lens facetado por país de la parte). Falta: lista CPC + ventana de ILIA 2025 (decisión: replicar).</t>
         </is>
       </c>
     </row>
@@ -3080,17 +3080,17 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Decisiones metodológicas</t>
+          <t>Decisiones metodológicas (estado)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>UE / SG</t>
+          <t>UE/SG/EE</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>(a) cómo puntuar el EU AI Act como 'iniciativa legal' en países UE; (b) si el Update SG may-2026 cambia 'Antigüedad'; (c) confirmar ISO SC42 de Estonia (=0).</t>
+          <t>RESUELTO 2026-06-16: EU AI Act=iniciativa legal (128=3); SG Antigüedad (104)=4 (Update may-2026); ERNC=renovables total; patentes 83=solicitante/84=inventor. PENDIENTE: confirmar ISO SC42 Estonia (=0) en iso.org; lista CPC+ventana de patentes de ILIA 2025.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Estonia validada con texto primario (Valge raamat + Tegevuskava)
Parseados los 2 PDF oficiales (White Paper 2024-2030, 56 pp; Tegevuskava 2024-2026,
47 pp) con PyMuPDF; codificación verbatim por subindicador. Quita el estado PRELIM de
Estonia. Dos cambios de puntaje:
- Sostenibilidad (118): 1 (BAJA) -> 0 (no es eje/área de acción; "kestlik areng" = econ.
  de datos, no ambiental). ⚠️ reversible si ILIA define "Sostenibilidad" en sentido amplio.
- Multistakeholder elaboración (121): 3 -> 4 (Gob+3: ITL/empresas + universidades +
  vabaühendused, p.8/12).
Confirmados (sin cambio): 103-108, 119(=2), 122(=4), 123-124, 128-130 (sandbox nacional
propio, p.52); género 117=0 confirmado (solo métrica, p.30).
- gobernanza/VALIDACION_estonia_primaria.md: citas textuales por tópico (109-118) + tabla
  de cambios. Cobertura ahora 143 verde / 16 ámbar / 31 rojo. Regenerados todos los
  entregables (planilla, PDF, por_pais, resumen).

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
+++ b/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
@@ -1399,9 +1399,9 @@
           <t>Estrategia</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>3 (PRELIM)</t>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -1875,9 +1875,9 @@
           <t>Estrategia</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>1 (BAJA)</t>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>PT: solo principio en EDN, no eje en ANIA</t>
+          <t>EE: validado en Valge raamat (no es eje; 'kestlik areng' = econ. de datos); PT: solo principio en EDN, no eje en ANIA</t>
         </is>
       </c>
     </row>
@@ -1918,9 +1918,9 @@
           <t>Estrategia</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>2 (PRELIM)</t>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>PT: consulta pública con resultados</t>
+          <t>EE: stakeholders ('Kaasatud osapooled'), no consulta ciudadana; PT: consulta pública con resultados</t>
         </is>
       </c>
     </row>
@@ -1961,16 +1961,16 @@
           <t>Estrategia</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>3 (PRELIM)</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>3 (PRELIM)</t>
-        </is>
-      </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
           <t>4 (PRELIM)</t>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>PT: Gob+4</t>
+          <t>EE: Gob+3 (ITL/empresas + universidades + vabaühendused), p.8/12; PT: Gob+4</t>
         </is>
       </c>
     </row>
@@ -2004,9 +2004,9 @@
           <t>Estrategia</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>4 (PRELIM)</t>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Estonia: Participación ciudadana (119) 4->5 (>1 mecanismo)
Corrección metodológica del operador: 119 mide MECANISMOS de participación y 121 mide
CUÁNTOS SECTORES; son ejes ortogonales (no hay doble conteo). En la elaboración hubo
>1 mecanismo con resultados publicados: 2 encuestas ómnibus (2150 residentes) + 220
kaasamisintervjuud (Tegevuskava p.6; resultado "77% ... suhtub pigem positiivselt",
Valge raamat p.44) -> 119 = 5. El nº de sectores (Gob+3) sigue en 121 = 4.
Actualizados G, detalle, VALIDACION y HANDOFF; regenerado todo. Cobertura 143/16/31.

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
+++ b/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
@@ -1920,32 +1920,32 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>1 (PRELIM)</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>3 (PRELIM)</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>1 (PRELIM)</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>3 (PRELIM)</t>
-        </is>
-      </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>EE: 2 encuestas ómnibus (2150 residentes) + 220 entrevistas, resultados publicados; PT: consulta pública con resultados</t>
+          <t>EE: &gt;1 mecanismo (2 encuestas ómnibus 2150 residentes + 220 entrevistas), resultados publicados; PT: consulta pública con resultados</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Estonia: Multistakeholder elaboración (121) 4->5 (Gob+4: ONG + público general)
Criterio del operador: contar ONG sin fines de lucro y público general como sectores
distintos. El texto primario respalda ambos en la ELABORACIÓN:
- ONG: vabaühendused (Valge raamat p.8) + 66 MTÜ en el ecosistema X-tee (p.51).
- Público general: 2150 residentes en 2 encuestas ómnibus + 220 entrevistas (PA p.6);
  el VR incorpora "kodaniku perspektiive" (p.8).
→ Gob+4 = 5. (Salvedad documentada: si el 4º sector ILIA = organismos internacionales,
sería 4.) Sin cambio de color (143/16/31). 122 sin cambiar (pendiente decisión 3 vs 4).

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
+++ b/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>EE: Gob+3 (ITL/empresas + universidades + vabaühendused), p.8/12; PT: Gob+4</t>
+          <t>EE: Gob+4 (privado + academia + ONG vabaühendused + público general/encuestas 2150), p.8/12 + PA p.6; PT: Gob+4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Indicador 145: energía limpia = renovables + nuclear (incl. hidro), EMBER 2025
Decisión del operador (a confirmar con CENIA): contar como "energía limpia" las
renovables + nuclear, incluyendo toda la hidro, con datos EMBER 2025 directos.
- ember_generacion_electrica_2025.csv (fuente versionada) + energia_limpia_ember2025.py
  (cálculo determinístico reproducible) + energia_limpia_resultados_2025.csv.
- Valores 145: ES 74,65% (renov 55,86 + nuclear 18,79) · EE 60,26% · SG 5,49% ·
  DE 59,09% · PT 80,90%. Solo España tiene nuclear.
- Actualizados G, GOBDET (x5) y HANDOFF (§3/§7). Regenerado todo. Cobertura 143/16/31.

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
+++ b/data/paises_extra/Planilla_ILIA2026_paises_extra.xlsx
@@ -2798,37 +2798,37 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>EMBER</t>
+          <t>EMBER 2025</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>55,75%</t>
+          <t>60,26%</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
         <is>
-          <t>4,93%</t>
+          <t>5,49%</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>58,64%</t>
+          <t>59,09%</t>
         </is>
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>57,34%</t>
+          <t>74,65%</t>
         </is>
       </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
-          <t>85,19%</t>
+          <t>80,90%</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>2024, renovables total. ES/PT/DE: ERNC excl. gran hidro es menor (ver energia_*.md)</t>
+          <t>Energía limpia = renovables + NUCLEAR (incl. hidro). EMBER 2025, determinístico (energia_limpia_ember2025.py). Solo ES tiene nuclear (18,79%). A confirmar con CENIA</t>
         </is>
       </c>
     </row>

</xml_diff>